<commit_message>
vault: sync 4 file(s) — 2026-05-28 19:51
</commit_message>
<xml_diff>
--- a/brantham/deals/active/open-bee-france/dataroom/open-bee-data-reelle-csv/Open bees .xlsx
+++ b/brantham/deals/active/open-bee-france/dataroom/open-bee-data-reelle-csv/Open bees .xlsx
@@ -8,13 +8,33 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paul/vault/brantham/deals/active/open-bee-france/dataroom/open-bee-data-reelle-csv/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC410034-B0D7-3E49-9909-E2912FDE98A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10EB0605-B22A-CA41-9852-CF09710D7FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{950FC21C-00BA-F04E-9B17-9E2A9235A7BD}"/>
+    <workbookView minimized="1" xWindow="20" yWindow="660" windowWidth="30240" windowHeight="17680" xr2:uid="{950FC21C-00BA-F04E-9B17-9E2A9235A7BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Feuil1!$B$69:$B$74</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Feuil1!$C$68</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">Feuil1!$C$68</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">Feuil1!$C$69:$C$74</definedName>
+    <definedName name="_xlchart.v1.12" hidden="1">Feuil1!$D$68</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">Feuil1!$D$69:$D$74</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">Feuil1!$E$68</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">Feuil1!$E$69:$E$74</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">Feuil1!$F$68</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">Feuil1!$F$69:$F$74</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Feuil1!$C$69:$C$74</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Feuil1!$D$68</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Feuil1!$D$69:$D$74</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Feuil1!$E$68</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Feuil1!$E$69:$E$74</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Feuil1!$F$68</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Feuil1!$F$69:$F$74</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Feuil1!$B$69:$B$74</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="68">
   <si>
     <t xml:space="preserve">Open Bee France (M€) </t>
   </si>
@@ -138,6 +158,206 @@
   </si>
   <si>
     <t>Q325</t>
+  </si>
+  <si>
+    <t>en M€</t>
+  </si>
+  <si>
+    <t>3Q25</t>
+  </si>
+  <si>
+    <t>Tréso. dispo.</t>
+  </si>
+  <si>
+    <t>Var. vs point préc.</t>
+  </si>
+  <si>
+    <t>CA FY24</t>
+  </si>
+  <si>
+    <t>RN FY24</t>
+  </si>
+  <si>
+    <t>Dév.capitalisés</t>
+  </si>
+  <si>
+    <t>Trésorerie</t>
+  </si>
+  <si>
+    <t>Dette fin. Brute</t>
+  </si>
+  <si>
+    <t>Priorité</t>
+  </si>
+  <si>
+    <t>Constat pré-RJ</t>
+  </si>
+  <si>
+    <t>Levier repreneur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA transféré à securiser </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2,01M€</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> à normaliser </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Normaliser </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base de coûts à rebaser </t>
+  </si>
+  <si>
+    <t>Actifs utiles à conserver</t>
+  </si>
+  <si>
+    <t>BFR post-reprise à calibrer</t>
+  </si>
+  <si>
+    <t>Passif à isoler</t>
+  </si>
+  <si>
+    <t>Repartir sur base saine</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">1,59M€ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">à retraiter </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1,29M€</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> à tester </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0,02M€ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">disponible </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4,39M€</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> historique </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Périmètre </t>
+  </si>
+  <si>
+    <t>Logi. GED/IP</t>
+  </si>
+  <si>
+    <t>Clients &amp; contrats</t>
+  </si>
+  <si>
+    <t>Partenaires</t>
+  </si>
+  <si>
+    <t>Équipe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facturation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrats </t>
+  </si>
+  <si>
+    <t>Reprendre</t>
+  </si>
+  <si>
+    <t>Reprendre sous condition</t>
+  </si>
+  <si>
+    <t>Laisser procédure</t>
+  </si>
+  <si>
+    <t>Priorité stratégique</t>
   </si>
 </sst>
 </file>
@@ -147,10 +367,17 @@
   <numFmts count="1">
     <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -169,7 +396,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -182,8 +409,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF55759B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0B1D3A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -202,36 +441,45 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
@@ -255,10 +503,34 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="17" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -267,9 +539,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF55759B"/>
+      <color rgb="FF4EC7C2"/>
+      <color rgb="FF91A9C2"/>
       <color rgb="FF0B1D3A"/>
       <color rgb="FFB9C9D9"/>
-      <color rgb="FF55759B"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1146,6 +1420,565 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Feuil1!$C$68</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Reprendre</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0B1D3A"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Feuil1!$B$69:$B$74</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Logi. GED/IP</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Clients &amp; contrats</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Partenaires</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Équipe</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Facturation </c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Contrats </c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Feuil1!$C$69:$C$74</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>65</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F1FE-6843-85E0-5EA8BC557AB4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Feuil1!$D$68</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Reprendre sous condition</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="91A9C2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Feuil1!$B$69:$B$74</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Logi. GED/IP</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Clients &amp; contrats</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Partenaires</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Équipe</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Facturation </c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Contrats </c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Feuil1!$D$69:$D$74</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>30</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-F1FE-6843-85E0-5EA8BC557AB4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Feuil1!$E$68</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Laisser procédure</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Feuil1!$B$69:$B$74</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Logi. GED/IP</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Clients &amp; contrats</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Partenaires</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Équipe</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Facturation </c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Contrats </c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Feuil1!$E$69:$E$74</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-F1FE-6843-85E0-5EA8BC557AB4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="115"/>
+        <c:overlap val="100"/>
+        <c:axId val="789382463"/>
+        <c:axId val="978725375"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Feuil1!$F$68</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Priorité stratégique</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="55759B"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Feuil1!$B$69:$B$74</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Logi. GED/IP</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Clients &amp; contrats</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Partenaires</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Équipe</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Facturation </c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Contrats </c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Feuil1!$F$69:$F$74</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>35</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-F1FE-6843-85E0-5EA8BC557AB4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="789382463"/>
+        <c:axId val="978725375"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="789382463"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="978725375"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="978725375"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="789382463"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="25400">
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1226,6 +2059,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
   <cs:axisTitle>
@@ -2215,6 +3088,522 @@
             <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -2259,8 +3648,8 @@
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>139700</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>134155</xdr:rowOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>47317</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2303,8 +3692,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>352985</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>114680</xdr:rowOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>129015</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2417,10 +3806,10 @@
       <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>10160</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>200660</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>706415</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>2223</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2451,6 +3840,174 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>415841</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>157345</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>390838</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>72940</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Image 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{41E35FA7-2F7A-BB68-2A8F-891F1A8C4160}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17645133" y="8653982"/>
+          <a:ext cx="4330700" cy="927100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>504757</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>23779</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>407391</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>49179</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Image 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{08BA082E-44FE-4FC9-E32E-0EE5429B85BA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22256885" y="1266758"/>
+          <a:ext cx="7036251" cy="2097031"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>668867</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>110067</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>135467</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>136107</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Image 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1E041CE6-2629-C095-8A1D-0835EECA06B4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1507067" y="12327467"/>
+          <a:ext cx="7848600" cy="1245240"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>199571</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>147865</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>644071</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>97064</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="22" name="Graphique 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{38E3C5D3-06C1-AA5E-B0BB-CEE5D6474A2E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -2773,10 +4330,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F77AF0FA-BE78-804F-BA51-924B1E1FDF3C}">
-  <dimension ref="B4:Q44"/>
+  <dimension ref="B4:AD74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="20" max="20" width="24.33203125" customWidth="1"/>
+    <col min="21" max="21" width="20.83203125" customWidth="1"/>
+    <col min="22" max="22" width="25.1640625" customWidth="1"/>
+    <col min="27" max="27" width="17.5" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
         <v>0</v>
       </c>
@@ -2790,7 +4353,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B5" s="6" t="s">
         <v>4</v>
       </c>
@@ -2808,7 +4371,7 @@
         <v>+40,8%</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>5</v>
       </c>
@@ -2823,7 +4386,7 @@
         <v>+34,3%</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>6</v>
       </c>
@@ -2837,8 +4400,14 @@
         <f>"+1,2%"</f>
         <v>+1,2%</v>
       </c>
+      <c r="U7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="V7" s="3" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>7</v>
       </c>
@@ -2852,8 +4421,17 @@
         <f>"+12,8%"</f>
         <v>+12,8%</v>
       </c>
+      <c r="T8" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="U8" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="V8" s="31" t="s">
+        <v>45</v>
+      </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B9" s="10" t="s">
         <v>8</v>
       </c>
@@ -2869,8 +4447,17 @@
       <c r="H9" s="12" t="s">
         <v>10</v>
       </c>
+      <c r="T9" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="U9" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="V9" s="29" t="s">
+        <v>48</v>
+      </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B10" s="6" t="s">
         <v>9</v>
       </c>
@@ -2886,13 +4473,31 @@
       <c r="H10" s="8" t="s">
         <v>10</v>
       </c>
+      <c r="T10" t="s">
+        <v>39</v>
+      </c>
+      <c r="U10" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="V10" s="1" t="s">
+        <v>49</v>
+      </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:22" x14ac:dyDescent="0.2">
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
+      <c r="T11" t="s">
+        <v>40</v>
+      </c>
+      <c r="U11" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="V11" s="1" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B12" s="16" t="s">
         <v>11</v>
       </c>
@@ -2909,8 +4514,17 @@
         <f>"-16,6 pt"</f>
         <v>-16,6 pt</v>
       </c>
+      <c r="T12" t="s">
+        <v>41</v>
+      </c>
+      <c r="U12" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="V12" s="1" t="s">
+        <v>51</v>
+      </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B13" s="13" t="s">
         <v>12</v>
       </c>
@@ -2926,8 +4540,17 @@
       <c r="H13" s="15">
         <v>-0.32100000000000001</v>
       </c>
+      <c r="T13" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="U13" s="29" t="s">
+        <v>47</v>
+      </c>
+      <c r="V13" s="29" t="s">
+        <v>52</v>
+      </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B14" s="16" t="s">
         <v>13</v>
       </c>
@@ -2944,7 +4567,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
         <v>19</v>
       </c>
@@ -2959,7 +4582,7 @@
       </c>
       <c r="G22" s="1"/>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>22</v>
       </c>
@@ -2974,7 +4597,7 @@
       </c>
       <c r="G23" s="3"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:30" ht="7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
         <v>17</v>
       </c>
@@ -2989,7 +4612,7 @@
       </c>
       <c r="G24" s="3"/>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:30" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
         <v>21</v>
       </c>
@@ -3003,8 +4626,20 @@
         <v>0.20699999999999999</v>
       </c>
       <c r="G25" s="3"/>
+      <c r="AA25" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB25" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC25" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD25" s="3" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:30" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>24</v>
       </c>
@@ -3018,8 +4653,20 @@
         <v>9.2999999999999999E-2</v>
       </c>
       <c r="G26" s="3"/>
+      <c r="AA26" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB26" s="1">
+        <v>0.47</v>
+      </c>
+      <c r="AC26" s="1">
+        <v>1.52</v>
+      </c>
+      <c r="AD26" s="1">
+        <v>0.02</v>
+      </c>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:30" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
         <v>18</v>
       </c>
@@ -3033,8 +4680,21 @@
         <v>1.2E-2</v>
       </c>
       <c r="G27" s="3"/>
+      <c r="AA27" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB27" s="1">
+        <v>-0.22</v>
+      </c>
+      <c r="AC27" s="1" t="str">
+        <f>"+1,05"</f>
+        <v>+1,05</v>
+      </c>
+      <c r="AD27" s="1">
+        <v>-1.5</v>
+      </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
         <v>23</v>
       </c>
@@ -3049,14 +4709,14 @@
       </c>
       <c r="G28" s="3"/>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:30" x14ac:dyDescent="0.2">
       <c r="B29" s="2"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
       <c r="F29" s="22"/>
       <c r="G29" s="3"/>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:30" x14ac:dyDescent="0.2">
       <c r="F30" s="19"/>
     </row>
     <row r="38" spans="16:17" x14ac:dyDescent="0.2">
@@ -3113,6 +4773,125 @@
       </c>
       <c r="Q44">
         <v>1.9E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B68" t="s">
+        <v>57</v>
+      </c>
+      <c r="C68" t="s">
+        <v>64</v>
+      </c>
+      <c r="D68" t="s">
+        <v>65</v>
+      </c>
+      <c r="E68" t="s">
+        <v>66</v>
+      </c>
+      <c r="F68" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B69" t="s">
+        <v>58</v>
+      </c>
+      <c r="C69">
+        <v>100</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="70" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B70" t="s">
+        <v>59</v>
+      </c>
+      <c r="C70">
+        <v>85</v>
+      </c>
+      <c r="D70">
+        <v>15</v>
+      </c>
+      <c r="E70">
+        <v>0</v>
+      </c>
+      <c r="F70">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="71" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B71" t="s">
+        <v>60</v>
+      </c>
+      <c r="C71">
+        <v>80</v>
+      </c>
+      <c r="D71">
+        <v>20</v>
+      </c>
+      <c r="E71">
+        <v>0</v>
+      </c>
+      <c r="F71">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="72" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B72" t="s">
+        <v>61</v>
+      </c>
+      <c r="C72">
+        <v>65</v>
+      </c>
+      <c r="D72">
+        <v>25</v>
+      </c>
+      <c r="E72">
+        <v>10</v>
+      </c>
+      <c r="F72">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="73" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B73" t="s">
+        <v>62</v>
+      </c>
+      <c r="C73">
+        <v>60</v>
+      </c>
+      <c r="D73">
+        <v>40</v>
+      </c>
+      <c r="E73">
+        <v>0</v>
+      </c>
+      <c r="F73">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="74" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B74" t="s">
+        <v>63</v>
+      </c>
+      <c r="C74">
+        <v>20</v>
+      </c>
+      <c r="D74">
+        <v>30</v>
+      </c>
+      <c r="E74">
+        <v>50</v>
+      </c>
+      <c r="F74">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>